<commit_message>
Añadir actividad: Firma de Convienio con IAPG
</commit_message>
<xml_diff>
--- a/agenda_territorial_consolidada.xlsx
+++ b/agenda_territorial_consolidada.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q25"/>
+  <dimension ref="A1:Q26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1973,7 +1973,11 @@
           <t>Alto Valle</t>
         </is>
       </c>
-      <c r="O22" t="inlineStr"/>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>Sin especificar</t>
+        </is>
+      </c>
       <c r="P22" t="inlineStr">
         <is>
           <t>Jornada de integración y paneles provinciales compuestas por visitas a sitios estratégicos para el desarrollo de la provincia, encuentros con funcionarias/os y referentes locales y actividades de integración grupal con los participantes de la formación Gestión para el Desarrollo.</t>
@@ -2032,7 +2036,11 @@
           <t>Alto Valle</t>
         </is>
       </c>
-      <c r="O23" t="inlineStr"/>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>Sin especificar</t>
+        </is>
+      </c>
       <c r="P23" t="inlineStr">
         <is>
           <t>Jornada de integración y paneles provinciales compuestas por visitas a sitios estratégicos para el desarrollo de la provincia, encuentros con funcionarias/os y referentes locales y actividades de integración grupal con los participantes de la formación Gestión para el Desarrollo.</t>
@@ -2131,7 +2139,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr"/>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
       <c r="I25" t="inlineStr">
         <is>
           <t>ALTA</t>
@@ -2164,6 +2176,61 @@
         <v>100</v>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>34</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Firma de Convienio con IAPG</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>IAPG | SEEyA | Ministerio de Educación y DDHH</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>General Roca</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>CET 1</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr"/>
+      <c r="Q26" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Añadir actividad: YPF por ONU HABITAT
</commit_message>
<xml_diff>
--- a/agenda_territorial_consolidada.xlsx
+++ b/agenda_territorial_consolidada.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q26"/>
+  <dimension ref="A1:Q27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2231,6 +2231,61 @@
         <v>50</v>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>35</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>YPF por ONU HABITAT</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>YPF | ONU-Hábitat | Secretaría de Ambiente | UNRN-Arquitectura</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>Sin especificar</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>General Roca</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>UNRN</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr"/>
+      <c r="Q27" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Añadir actividad: Maquetas V4LE
</commit_message>
<xml_diff>
--- a/agenda_territorial_consolidada.xlsx
+++ b/agenda_territorial_consolidada.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q27"/>
+  <dimension ref="A1:Q28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2286,6 +2286,57 @@
         <v>50</v>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>37</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Maquetas V4LE</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>Sin especificar</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>Cipolletti</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr"/>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>Capacitación para el armado y el uso de las Maquetas V4LE.</t>
+        </is>
+      </c>
+      <c r="Q28" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>